<commit_message>
Video név lekérése - tárgy
</commit_message>
<xml_diff>
--- a/sablonok/EM-X.Y.Z-Formaiell.xlsx
+++ b/sablonok/EM-X.Y.Z-Formaiell.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oLovasz\MyRobotFramework\SandboxRobots\IKK-Robotok\IKK04-Dokumentum-WEB-Ellenőrzés\sablonok\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F640629-5C0A-46F3-9E92-27451DD7F305}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4EAA338-33BB-497A-80F4-E05652D12B9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28320" yWindow="2190" windowWidth="17280" windowHeight="14370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Alapadatok" sheetId="1" r:id="rId1"/>
@@ -236,12 +236,6 @@
     <t>Médiakredit érték</t>
   </si>
   <si>
-    <t>Vállalkozó által leadott adatok</t>
-  </si>
-  <si>
-    <t>Fájlnév (vállalkozótól)</t>
-  </si>
-  <si>
     <t>Médiaelem típusa</t>
   </si>
   <si>
@@ -261,6 +255,12 @@
   </si>
   <si>
     <t>Leírása</t>
+  </si>
+  <si>
+    <t>Robot által talált adatok</t>
+  </si>
+  <si>
+    <t>Fájlnév (robottól)</t>
   </si>
 </sst>
 </file>
@@ -1690,7 +1690,7 @@
       <c r="AA3" s="36"/>
       <c r="AB3" s="36"/>
     </row>
-    <row r="4" spans="1:28" s="25" customFormat="1" ht="120" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:28" s="25" customFormat="1" ht="105" x14ac:dyDescent="0.35">
       <c r="A4" s="40" t="s">
         <v>21</v>
       </c>
@@ -30361,7 +30361,7 @@
     </row>
     <row r="3" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="73" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="B3" s="74"/>
       <c r="C3" s="75"/>
@@ -30375,29 +30375,29 @@
     </row>
     <row r="4" spans="1:14" ht="45.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="76" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="78" t="s">
         <v>44</v>
       </c>
-      <c r="B4" s="77" t="s">
+      <c r="D4" s="79" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="78" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" s="79" t="s">
-        <v>47</v>
-      </c>
       <c r="E4" s="88" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F4" s="80"/>
       <c r="I4" s="81" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="J4" s="81" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="K4" s="82" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="L4" s="111"/>
     </row>

</xml_diff>

<commit_message>
Kapott média kezelés hiány jelzése sumError.csv-ben is
</commit_message>
<xml_diff>
--- a/sablonok/EM-X.Y.Z-Formaiell.xlsx
+++ b/sablonok/EM-X.Y.Z-Formaiell.xlsx
@@ -8,20 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oLovasz\MyRobotFramework\SandboxRobots\IKK-Robotok\IKK04-Dokumentum-WEB-Ellenőrzés\sablonok\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4EAA338-33BB-497A-80F4-E05652D12B9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AFE2266-EFE2-4A9E-A8A9-73C088F2A2E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Alapadatok" sheetId="1" r:id="rId1"/>
     <sheet name="EM-X.Y.Z" sheetId="5" r:id="rId2"/>
-    <sheet name="EM-X.Y.Z-MK" sheetId="7" r:id="rId3"/>
-    <sheet name="Médiatípusok" sheetId="3" r:id="rId4"/>
+    <sheet name="Médiatípusok" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'EM-X.Y.Z-MK'!$A$1:$G$4</definedName>
     <definedName name="Médiaelem_típusa" localSheetId="1">#REF!</definedName>
-    <definedName name="Médiaelem_típusa" localSheetId="2">#REF!</definedName>
     <definedName name="Médiaelem_típusa">Médiatípusok!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -42,44 +39,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Szücs Dániel</author>
-  </authors>
-  <commentList>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{A658620E-5A9F-4AFE-8FD3-98DCAA4B7A0D}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-            <charset val="238"/>
-          </rPr>
-          <t>Szücs Dániel:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-            <charset val="238"/>
-          </rPr>
-          <t xml:space="preserve">
-A nettó kéziratnak az oldalszáma</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>I/R</t>
   </si>
@@ -214,60 +175,12 @@
   <si>
     <t>-</t>
   </si>
-  <si>
-    <t>Médiakredit</t>
-  </si>
-  <si>
-    <t>darab</t>
-  </si>
-  <si>
-    <t>oldalszám:</t>
-  </si>
-  <si>
-    <t>A borászati üzemek jellemzői és a borászati termékek</t>
-  </si>
-  <si>
-    <t>interaktívitási szint:</t>
-  </si>
-  <si>
-    <t>Megtalálható a digitális tananyagban</t>
-  </si>
-  <si>
-    <t>Médiakredit érték</t>
-  </si>
-  <si>
-    <t>Médiaelem típusa</t>
-  </si>
-  <si>
-    <t>Lecke címe</t>
-  </si>
-  <si>
-    <t>Oldalcím</t>
-  </si>
-  <si>
-    <t>igen</t>
-  </si>
-  <si>
-    <t>nem</t>
-  </si>
-  <si>
-    <t>Mozgókép hossza (mp)</t>
-  </si>
-  <si>
-    <t>Leírása</t>
-  </si>
-  <si>
-    <t>Robot által talált adatok</t>
-  </si>
-  <si>
-    <t>Fájlnév (robottól)</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -341,82 +254,16 @@
       <family val="2"/>
       <charset val="238"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="238"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="238"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="238"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FF0070C0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="238"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-      <charset val="238"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-      <charset val="238"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="43">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -869,117 +716,15 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="6">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1157,82 +902,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="4" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="4" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="4" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="4"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="4" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="4" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="4" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="38" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="39" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="40" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="11" fillId="3" borderId="41" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="4" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="42" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1266,45 +935,8 @@
     <xf numFmtId="49" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="17" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="34" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="35" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="18" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="19" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="36" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="20" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="37" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="21" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="40" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="6">
-    <cellStyle name="Hivatkozás" xfId="5" builtinId="8"/>
+  <cellStyles count="5">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
     <cellStyle name="Normál 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Normál 2 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
@@ -1536,24 +1168,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="91" t="s">
+      <c r="A1" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="89" t="s">
+      <c r="C1" s="61" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="89" t="s">
+      <c r="D1" s="61" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="93"/>
+      <c r="E1" s="65"/>
     </row>
     <row r="2" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="92"/>
-      <c r="B2" s="90"/>
-      <c r="C2" s="90"/>
+      <c r="A2" s="64"/>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
       <c r="D2" s="3" t="s">
         <v>5</v>
       </c>
@@ -1609,9 +1241,9 @@
       <c r="A1" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="96"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="68"/>
       <c r="E1" s="53"/>
       <c r="F1" s="23"/>
       <c r="G1" s="24"/>
@@ -1988,11 +1620,11 @@
       <c r="A14" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="97" t="s">
+      <c r="B14" s="69" t="s">
         <v>35</v>
       </c>
-      <c r="C14" s="98"/>
-      <c r="D14" s="99"/>
+      <c r="C14" s="70"/>
+      <c r="D14" s="71"/>
       <c r="E14" s="59"/>
       <c r="F14" s="28"/>
       <c r="G14" s="28"/>
@@ -30294,1887 +29926,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73980D9D-1A52-475B-B6D6-7EF2F269935B}">
-  <dimension ref="A1:N591"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="34.59765625" style="67" customWidth="1"/>
-    <col min="2" max="2" width="13.5" style="67" customWidth="1"/>
-    <col min="3" max="3" width="20.59765625" style="85" customWidth="1"/>
-    <col min="4" max="5" width="20.69921875" style="85" customWidth="1"/>
-    <col min="6" max="6" width="14.5" style="85" customWidth="1"/>
-    <col min="7" max="7" width="9" style="67"/>
-    <col min="8" max="8" width="37.19921875" style="67" customWidth="1"/>
-    <col min="9" max="9" width="9" style="68"/>
-    <col min="10" max="10" width="9" style="67"/>
-    <col min="11" max="11" width="10.5" style="69" customWidth="1"/>
-    <col min="12" max="12" width="10.5" style="67" customWidth="1"/>
-    <col min="13" max="13" width="9" style="67"/>
-    <col min="14" max="14" width="48.8984375" style="67" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="9" style="67"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:14" ht="33.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="61" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="63" t="s">
-        <v>37</v>
-      </c>
-      <c r="D1" s="64">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
-      </c>
-      <c r="E1" s="86"/>
-      <c r="F1" s="65" t="s">
-        <v>38</v>
-      </c>
-      <c r="G1" s="66">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="70" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="100" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" s="101"/>
-      <c r="D2" s="102"/>
-      <c r="E2" s="87"/>
-      <c r="F2" s="71" t="s">
-        <v>40</v>
-      </c>
-      <c r="G2" s="72">
-        <v>5</v>
-      </c>
-      <c r="I2" s="103" t="s">
-        <v>41</v>
-      </c>
-      <c r="J2" s="104"/>
-      <c r="K2" s="105"/>
-      <c r="L2" s="109" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="73" t="s">
-        <v>50</v>
-      </c>
-      <c r="B3" s="74"/>
-      <c r="C3" s="75"/>
-      <c r="D3" s="75"/>
-      <c r="E3" s="75"/>
-      <c r="F3" s="75"/>
-      <c r="I3" s="106"/>
-      <c r="J3" s="107"/>
-      <c r="K3" s="108"/>
-      <c r="L3" s="110"/>
-    </row>
-    <row r="4" spans="1:14" ht="45.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="76" t="s">
-        <v>51</v>
-      </c>
-      <c r="B4" s="77" t="s">
-        <v>43</v>
-      </c>
-      <c r="C4" s="78" t="s">
-        <v>44</v>
-      </c>
-      <c r="D4" s="79" t="s">
-        <v>45</v>
-      </c>
-      <c r="E4" s="88" t="s">
-        <v>49</v>
-      </c>
-      <c r="F4" s="80"/>
-      <c r="I4" s="81" t="s">
-        <v>46</v>
-      </c>
-      <c r="J4" s="81" t="s">
-        <v>47</v>
-      </c>
-      <c r="K4" s="82" t="s">
-        <v>48</v>
-      </c>
-      <c r="L4" s="111"/>
-    </row>
-    <row r="5" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N5" s="84"/>
-    </row>
-    <row r="6" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N6" s="84"/>
-    </row>
-    <row r="7" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N7" s="84"/>
-    </row>
-    <row r="8" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N8" s="84"/>
-    </row>
-    <row r="9" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N9" s="84"/>
-    </row>
-    <row r="10" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N10" s="84"/>
-    </row>
-    <row r="11" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N11" s="84"/>
-    </row>
-    <row r="12" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N12" s="84"/>
-    </row>
-    <row r="13" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N13" s="84"/>
-    </row>
-    <row r="14" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N14" s="84"/>
-    </row>
-    <row r="15" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N15" s="84"/>
-    </row>
-    <row r="16" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N16" s="84"/>
-    </row>
-    <row r="17" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N17" s="84"/>
-    </row>
-    <row r="18" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N18" s="84"/>
-    </row>
-    <row r="19" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N19" s="84"/>
-    </row>
-    <row r="20" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N20" s="84"/>
-    </row>
-    <row r="21" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N21" s="84"/>
-    </row>
-    <row r="22" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N22" s="84"/>
-    </row>
-    <row r="23" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N23" s="84"/>
-    </row>
-    <row r="24" spans="14:14" x14ac:dyDescent="0.3">
-      <c r="N24" s="83"/>
-    </row>
-    <row r="25" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N25" s="84"/>
-    </row>
-    <row r="26" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N26" s="84"/>
-    </row>
-    <row r="27" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N27" s="84"/>
-    </row>
-    <row r="28" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N28" s="84"/>
-    </row>
-    <row r="29" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N29" s="84"/>
-    </row>
-    <row r="30" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N30" s="84"/>
-    </row>
-    <row r="31" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N31" s="84"/>
-    </row>
-    <row r="32" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N32" s="84"/>
-    </row>
-    <row r="33" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N33" s="84"/>
-    </row>
-    <row r="34" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N34" s="84"/>
-    </row>
-    <row r="35" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N35" s="84"/>
-    </row>
-    <row r="36" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N36" s="84"/>
-    </row>
-    <row r="37" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N37" s="84"/>
-    </row>
-    <row r="38" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N38" s="84"/>
-    </row>
-    <row r="39" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N39" s="84"/>
-    </row>
-    <row r="40" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N40" s="84"/>
-    </row>
-    <row r="41" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N41" s="84"/>
-    </row>
-    <row r="42" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N42" s="84"/>
-    </row>
-    <row r="43" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N43" s="84"/>
-    </row>
-    <row r="44" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N44" s="84"/>
-    </row>
-    <row r="45" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N45" s="84"/>
-    </row>
-    <row r="46" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N46" s="84"/>
-    </row>
-    <row r="47" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N47" s="84"/>
-    </row>
-    <row r="48" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N48" s="84"/>
-    </row>
-    <row r="49" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N49" s="84"/>
-    </row>
-    <row r="50" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N50" s="84"/>
-    </row>
-    <row r="51" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N51" s="84"/>
-    </row>
-    <row r="52" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N52" s="84"/>
-    </row>
-    <row r="53" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N53" s="84"/>
-    </row>
-    <row r="54" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N54" s="84"/>
-    </row>
-    <row r="55" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N55" s="84"/>
-    </row>
-    <row r="56" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N56" s="84"/>
-    </row>
-    <row r="57" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N57" s="84"/>
-    </row>
-    <row r="58" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N58" s="84"/>
-    </row>
-    <row r="59" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N59" s="84"/>
-    </row>
-    <row r="60" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N60" s="84"/>
-    </row>
-    <row r="61" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N61" s="84"/>
-    </row>
-    <row r="62" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N62" s="84"/>
-    </row>
-    <row r="63" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N63" s="84"/>
-    </row>
-    <row r="64" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N64" s="84"/>
-    </row>
-    <row r="65" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N65" s="84"/>
-    </row>
-    <row r="66" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N66" s="84"/>
-    </row>
-    <row r="67" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N67" s="84"/>
-    </row>
-    <row r="68" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N68" s="84"/>
-    </row>
-    <row r="69" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N69" s="84"/>
-    </row>
-    <row r="70" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N70" s="84"/>
-    </row>
-    <row r="71" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N71" s="84"/>
-    </row>
-    <row r="72" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N72" s="84"/>
-    </row>
-    <row r="73" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N73" s="84"/>
-    </row>
-    <row r="74" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N74" s="84"/>
-    </row>
-    <row r="75" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N75" s="84"/>
-    </row>
-    <row r="76" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N76" s="84"/>
-    </row>
-    <row r="77" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N77" s="84"/>
-    </row>
-    <row r="78" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N78" s="84"/>
-    </row>
-    <row r="79" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N79" s="84"/>
-    </row>
-    <row r="80" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N80" s="84"/>
-    </row>
-    <row r="81" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N81" s="84"/>
-    </row>
-    <row r="82" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N82" s="84"/>
-    </row>
-    <row r="83" spans="14:14" x14ac:dyDescent="0.3">
-      <c r="N83" s="83"/>
-    </row>
-    <row r="84" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N84" s="84"/>
-    </row>
-    <row r="85" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N85" s="84"/>
-    </row>
-    <row r="86" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N86" s="84"/>
-    </row>
-    <row r="87" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N87" s="84"/>
-    </row>
-    <row r="88" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N88" s="84"/>
-    </row>
-    <row r="89" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N89" s="84"/>
-    </row>
-    <row r="90" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N90" s="84"/>
-    </row>
-    <row r="91" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N91" s="84"/>
-    </row>
-    <row r="92" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N92" s="84"/>
-    </row>
-    <row r="93" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N93" s="84"/>
-    </row>
-    <row r="94" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N94" s="84"/>
-    </row>
-    <row r="95" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N95" s="84"/>
-    </row>
-    <row r="96" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N96" s="84"/>
-    </row>
-    <row r="97" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N97" s="84"/>
-    </row>
-    <row r="98" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N98" s="84"/>
-    </row>
-    <row r="99" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N99" s="84"/>
-    </row>
-    <row r="100" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N100" s="84"/>
-    </row>
-    <row r="101" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N101" s="84"/>
-    </row>
-    <row r="102" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N102" s="84"/>
-    </row>
-    <row r="103" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N103" s="84"/>
-    </row>
-    <row r="104" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N104" s="84"/>
-    </row>
-    <row r="105" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N105" s="84"/>
-    </row>
-    <row r="106" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N106" s="84"/>
-    </row>
-    <row r="107" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N107" s="84"/>
-    </row>
-    <row r="108" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N108" s="84"/>
-    </row>
-    <row r="109" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N109" s="84"/>
-    </row>
-    <row r="110" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N110" s="84"/>
-    </row>
-    <row r="111" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N111" s="84"/>
-    </row>
-    <row r="112" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N112" s="84"/>
-    </row>
-    <row r="113" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N113" s="84"/>
-    </row>
-    <row r="114" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N114" s="84"/>
-    </row>
-    <row r="115" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N115" s="84"/>
-    </row>
-    <row r="116" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N116" s="84"/>
-    </row>
-    <row r="117" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N117" s="84"/>
-    </row>
-    <row r="118" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N118" s="84"/>
-    </row>
-    <row r="119" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N119" s="84"/>
-    </row>
-    <row r="120" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N120" s="84"/>
-    </row>
-    <row r="121" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N121" s="84"/>
-    </row>
-    <row r="122" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N122" s="84"/>
-    </row>
-    <row r="123" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N123" s="84"/>
-    </row>
-    <row r="124" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N124" s="84"/>
-    </row>
-    <row r="125" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N125" s="84"/>
-    </row>
-    <row r="126" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N126" s="84"/>
-    </row>
-    <row r="127" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N127" s="84"/>
-    </row>
-    <row r="128" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N128" s="84"/>
-    </row>
-    <row r="129" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N129" s="84"/>
-    </row>
-    <row r="130" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N130" s="84"/>
-    </row>
-    <row r="131" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N131" s="84"/>
-    </row>
-    <row r="132" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N132" s="84"/>
-    </row>
-    <row r="133" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N133" s="84"/>
-    </row>
-    <row r="134" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N134" s="84"/>
-    </row>
-    <row r="135" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N135" s="84"/>
-    </row>
-    <row r="136" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N136" s="84"/>
-    </row>
-    <row r="137" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N137" s="84"/>
-    </row>
-    <row r="138" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N138" s="84"/>
-    </row>
-    <row r="139" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N139" s="84"/>
-    </row>
-    <row r="140" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N140" s="84"/>
-    </row>
-    <row r="141" spans="14:14" x14ac:dyDescent="0.3">
-      <c r="N141" s="83"/>
-    </row>
-    <row r="142" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N142" s="84"/>
-    </row>
-    <row r="143" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N143" s="84"/>
-    </row>
-    <row r="144" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N144" s="84"/>
-    </row>
-    <row r="145" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N145" s="84"/>
-    </row>
-    <row r="146" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N146" s="84"/>
-    </row>
-    <row r="147" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N147" s="84"/>
-    </row>
-    <row r="148" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N148" s="84"/>
-    </row>
-    <row r="149" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N149" s="84"/>
-    </row>
-    <row r="150" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N150" s="84"/>
-    </row>
-    <row r="151" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N151" s="84"/>
-    </row>
-    <row r="152" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N152" s="84"/>
-    </row>
-    <row r="153" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N153" s="84"/>
-    </row>
-    <row r="154" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N154" s="84"/>
-    </row>
-    <row r="155" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N155" s="84"/>
-    </row>
-    <row r="156" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N156" s="84"/>
-    </row>
-    <row r="157" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N157" s="84"/>
-    </row>
-    <row r="158" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N158" s="84"/>
-    </row>
-    <row r="159" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N159" s="84"/>
-    </row>
-    <row r="160" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N160" s="84"/>
-    </row>
-    <row r="161" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N161" s="84"/>
-    </row>
-    <row r="162" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N162" s="84"/>
-    </row>
-    <row r="163" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N163" s="84"/>
-    </row>
-    <row r="164" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N164" s="84"/>
-    </row>
-    <row r="165" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N165" s="84"/>
-    </row>
-    <row r="166" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N166" s="84"/>
-    </row>
-    <row r="167" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N167" s="84"/>
-    </row>
-    <row r="168" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N168" s="84"/>
-    </row>
-    <row r="169" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N169" s="84"/>
-    </row>
-    <row r="170" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N170" s="84"/>
-    </row>
-    <row r="171" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N171" s="84"/>
-    </row>
-    <row r="172" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N172" s="84"/>
-    </row>
-    <row r="173" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N173" s="84"/>
-    </row>
-    <row r="174" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N174" s="84"/>
-    </row>
-    <row r="175" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N175" s="84"/>
-    </row>
-    <row r="176" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N176" s="84"/>
-    </row>
-    <row r="177" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N177" s="84"/>
-    </row>
-    <row r="178" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N178" s="84"/>
-    </row>
-    <row r="179" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N179" s="84"/>
-    </row>
-    <row r="180" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N180" s="84"/>
-    </row>
-    <row r="181" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N181" s="84"/>
-    </row>
-    <row r="182" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N182" s="84"/>
-    </row>
-    <row r="183" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N183" s="84"/>
-    </row>
-    <row r="184" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N184" s="84"/>
-    </row>
-    <row r="185" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N185" s="84"/>
-    </row>
-    <row r="186" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N186" s="84"/>
-    </row>
-    <row r="187" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N187" s="84"/>
-    </row>
-    <row r="188" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N188" s="84"/>
-    </row>
-    <row r="189" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N189" s="84"/>
-    </row>
-    <row r="190" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N190" s="84"/>
-    </row>
-    <row r="191" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N191" s="84"/>
-    </row>
-    <row r="192" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N192" s="84"/>
-    </row>
-    <row r="193" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N193" s="84"/>
-    </row>
-    <row r="194" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N194" s="84"/>
-    </row>
-    <row r="195" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N195" s="84"/>
-    </row>
-    <row r="196" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N196" s="84"/>
-    </row>
-    <row r="197" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N197" s="84"/>
-    </row>
-    <row r="198" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N198" s="84"/>
-    </row>
-    <row r="199" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N199" s="84"/>
-    </row>
-    <row r="200" spans="14:14" x14ac:dyDescent="0.3">
-      <c r="N200" s="83"/>
-    </row>
-    <row r="201" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N201" s="84"/>
-    </row>
-    <row r="202" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N202" s="84"/>
-    </row>
-    <row r="203" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N203" s="84"/>
-    </row>
-    <row r="204" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N204" s="84"/>
-    </row>
-    <row r="205" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N205" s="84"/>
-    </row>
-    <row r="206" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N206" s="84"/>
-    </row>
-    <row r="207" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N207" s="84"/>
-    </row>
-    <row r="208" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N208" s="84"/>
-    </row>
-    <row r="209" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N209" s="84"/>
-    </row>
-    <row r="210" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N210" s="84"/>
-    </row>
-    <row r="211" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N211" s="84"/>
-    </row>
-    <row r="212" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N212" s="84"/>
-    </row>
-    <row r="213" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N213" s="84"/>
-    </row>
-    <row r="214" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N214" s="84"/>
-    </row>
-    <row r="215" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N215" s="84"/>
-    </row>
-    <row r="216" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N216" s="84"/>
-    </row>
-    <row r="217" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N217" s="84"/>
-    </row>
-    <row r="218" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N218" s="84"/>
-    </row>
-    <row r="219" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N219" s="84"/>
-    </row>
-    <row r="220" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N220" s="84"/>
-    </row>
-    <row r="221" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N221" s="84"/>
-    </row>
-    <row r="222" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N222" s="84"/>
-    </row>
-    <row r="223" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N223" s="84"/>
-    </row>
-    <row r="224" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N224" s="84"/>
-    </row>
-    <row r="225" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N225" s="84"/>
-    </row>
-    <row r="226" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N226" s="84"/>
-    </row>
-    <row r="227" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N227" s="84"/>
-    </row>
-    <row r="228" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N228" s="84"/>
-    </row>
-    <row r="229" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N229" s="84"/>
-    </row>
-    <row r="230" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N230" s="84"/>
-    </row>
-    <row r="231" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N231" s="84"/>
-    </row>
-    <row r="232" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N232" s="84"/>
-    </row>
-    <row r="233" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N233" s="84"/>
-    </row>
-    <row r="234" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N234" s="84"/>
-    </row>
-    <row r="235" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N235" s="84"/>
-    </row>
-    <row r="236" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N236" s="84"/>
-    </row>
-    <row r="237" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N237" s="84"/>
-    </row>
-    <row r="238" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N238" s="84"/>
-    </row>
-    <row r="239" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N239" s="84"/>
-    </row>
-    <row r="240" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N240" s="84"/>
-    </row>
-    <row r="241" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N241" s="84"/>
-    </row>
-    <row r="242" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N242" s="84"/>
-    </row>
-    <row r="243" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N243" s="84"/>
-    </row>
-    <row r="244" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N244" s="84"/>
-    </row>
-    <row r="245" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N245" s="84"/>
-    </row>
-    <row r="246" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N246" s="84"/>
-    </row>
-    <row r="247" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N247" s="84"/>
-    </row>
-    <row r="248" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N248" s="84"/>
-    </row>
-    <row r="249" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N249" s="84"/>
-    </row>
-    <row r="250" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N250" s="84"/>
-    </row>
-    <row r="251" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N251" s="84"/>
-    </row>
-    <row r="252" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N252" s="84"/>
-    </row>
-    <row r="253" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N253" s="84"/>
-    </row>
-    <row r="254" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N254" s="84"/>
-    </row>
-    <row r="255" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N255" s="84"/>
-    </row>
-    <row r="256" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N256" s="84"/>
-    </row>
-    <row r="257" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N257" s="84"/>
-    </row>
-    <row r="258" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N258" s="84"/>
-    </row>
-    <row r="259" spans="14:14" x14ac:dyDescent="0.3">
-      <c r="N259" s="83"/>
-    </row>
-    <row r="260" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N260" s="84"/>
-    </row>
-    <row r="261" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N261" s="84"/>
-    </row>
-    <row r="262" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N262" s="84"/>
-    </row>
-    <row r="263" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N263" s="84"/>
-    </row>
-    <row r="264" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N264" s="84"/>
-    </row>
-    <row r="265" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N265" s="84"/>
-    </row>
-    <row r="266" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N266" s="84"/>
-    </row>
-    <row r="267" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N267" s="84"/>
-    </row>
-    <row r="268" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N268" s="84"/>
-    </row>
-    <row r="269" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N269" s="84"/>
-    </row>
-    <row r="270" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N270" s="84"/>
-    </row>
-    <row r="271" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N271" s="84"/>
-    </row>
-    <row r="272" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N272" s="84"/>
-    </row>
-    <row r="273" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N273" s="84"/>
-    </row>
-    <row r="274" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N274" s="84"/>
-    </row>
-    <row r="275" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N275" s="84"/>
-    </row>
-    <row r="276" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N276" s="84"/>
-    </row>
-    <row r="277" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N277" s="84"/>
-    </row>
-    <row r="278" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N278" s="84"/>
-    </row>
-    <row r="279" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N279" s="84"/>
-    </row>
-    <row r="280" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N280" s="84"/>
-    </row>
-    <row r="281" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N281" s="84"/>
-    </row>
-    <row r="282" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N282" s="84"/>
-    </row>
-    <row r="283" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N283" s="84"/>
-    </row>
-    <row r="284" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N284" s="84"/>
-    </row>
-    <row r="285" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N285" s="84"/>
-    </row>
-    <row r="286" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N286" s="84"/>
-    </row>
-    <row r="287" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N287" s="84"/>
-    </row>
-    <row r="288" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N288" s="84"/>
-    </row>
-    <row r="289" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N289" s="84"/>
-    </row>
-    <row r="290" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N290" s="84"/>
-    </row>
-    <row r="291" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N291" s="84"/>
-    </row>
-    <row r="292" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N292" s="84"/>
-    </row>
-    <row r="293" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N293" s="84"/>
-    </row>
-    <row r="294" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N294" s="84"/>
-    </row>
-    <row r="295" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N295" s="84"/>
-    </row>
-    <row r="296" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N296" s="84"/>
-    </row>
-    <row r="297" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N297" s="84"/>
-    </row>
-    <row r="298" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N298" s="84"/>
-    </row>
-    <row r="299" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N299" s="84"/>
-    </row>
-    <row r="300" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N300" s="84"/>
-    </row>
-    <row r="301" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N301" s="84"/>
-    </row>
-    <row r="302" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N302" s="84"/>
-    </row>
-    <row r="303" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N303" s="84"/>
-    </row>
-    <row r="304" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N304" s="84"/>
-    </row>
-    <row r="305" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N305" s="84"/>
-    </row>
-    <row r="306" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N306" s="84"/>
-    </row>
-    <row r="307" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N307" s="84"/>
-    </row>
-    <row r="308" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N308" s="84"/>
-    </row>
-    <row r="309" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N309" s="84"/>
-    </row>
-    <row r="310" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N310" s="84"/>
-    </row>
-    <row r="311" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N311" s="84"/>
-    </row>
-    <row r="312" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N312" s="84"/>
-    </row>
-    <row r="313" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N313" s="84"/>
-    </row>
-    <row r="314" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N314" s="84"/>
-    </row>
-    <row r="315" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N315" s="84"/>
-    </row>
-    <row r="316" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N316" s="84"/>
-    </row>
-    <row r="317" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N317" s="84"/>
-    </row>
-    <row r="318" spans="14:14" x14ac:dyDescent="0.3">
-      <c r="N318" s="83"/>
-    </row>
-    <row r="319" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N319" s="84"/>
-    </row>
-    <row r="320" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N320" s="84"/>
-    </row>
-    <row r="321" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N321" s="84"/>
-    </row>
-    <row r="322" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N322" s="84"/>
-    </row>
-    <row r="323" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N323" s="84"/>
-    </row>
-    <row r="324" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N324" s="84"/>
-    </row>
-    <row r="325" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N325" s="84"/>
-    </row>
-    <row r="326" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N326" s="84"/>
-    </row>
-    <row r="327" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N327" s="84"/>
-    </row>
-    <row r="328" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N328" s="84"/>
-    </row>
-    <row r="329" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N329" s="84"/>
-    </row>
-    <row r="330" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N330" s="84"/>
-    </row>
-    <row r="331" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N331" s="84"/>
-    </row>
-    <row r="332" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N332" s="84"/>
-    </row>
-    <row r="333" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N333" s="84"/>
-    </row>
-    <row r="334" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N334" s="84"/>
-    </row>
-    <row r="335" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N335" s="84"/>
-    </row>
-    <row r="336" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N336" s="84"/>
-    </row>
-    <row r="337" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N337" s="84"/>
-    </row>
-    <row r="338" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N338" s="84"/>
-    </row>
-    <row r="339" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N339" s="84"/>
-    </row>
-    <row r="340" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N340" s="84"/>
-    </row>
-    <row r="341" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N341" s="84"/>
-    </row>
-    <row r="342" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N342" s="84"/>
-    </row>
-    <row r="343" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N343" s="84"/>
-    </row>
-    <row r="344" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N344" s="84"/>
-    </row>
-    <row r="345" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N345" s="84"/>
-    </row>
-    <row r="346" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N346" s="84"/>
-    </row>
-    <row r="347" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N347" s="84"/>
-    </row>
-    <row r="348" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N348" s="84"/>
-    </row>
-    <row r="349" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N349" s="84"/>
-    </row>
-    <row r="350" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N350" s="84"/>
-    </row>
-    <row r="351" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N351" s="84"/>
-    </row>
-    <row r="352" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N352" s="84"/>
-    </row>
-    <row r="353" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N353" s="84"/>
-    </row>
-    <row r="354" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N354" s="84"/>
-    </row>
-    <row r="355" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N355" s="84"/>
-    </row>
-    <row r="356" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N356" s="84"/>
-    </row>
-    <row r="357" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N357" s="84"/>
-    </row>
-    <row r="358" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N358" s="84"/>
-    </row>
-    <row r="359" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N359" s="84"/>
-    </row>
-    <row r="360" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N360" s="84"/>
-    </row>
-    <row r="361" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N361" s="84"/>
-    </row>
-    <row r="362" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N362" s="84"/>
-    </row>
-    <row r="363" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N363" s="84"/>
-    </row>
-    <row r="364" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N364" s="84"/>
-    </row>
-    <row r="365" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N365" s="84"/>
-    </row>
-    <row r="366" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N366" s="84"/>
-    </row>
-    <row r="367" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N367" s="84"/>
-    </row>
-    <row r="368" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N368" s="84"/>
-    </row>
-    <row r="369" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N369" s="84"/>
-    </row>
-    <row r="370" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N370" s="84"/>
-    </row>
-    <row r="371" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N371" s="84"/>
-    </row>
-    <row r="372" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N372" s="84"/>
-    </row>
-    <row r="373" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N373" s="84"/>
-    </row>
-    <row r="374" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N374" s="84"/>
-    </row>
-    <row r="375" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N375" s="84"/>
-    </row>
-    <row r="376" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N376" s="84"/>
-    </row>
-    <row r="377" spans="14:14" x14ac:dyDescent="0.3">
-      <c r="N377" s="83"/>
-    </row>
-    <row r="378" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N378" s="84"/>
-    </row>
-    <row r="379" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N379" s="84"/>
-    </row>
-    <row r="380" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N380" s="84"/>
-    </row>
-    <row r="381" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N381" s="84"/>
-    </row>
-    <row r="382" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N382" s="84"/>
-    </row>
-    <row r="383" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N383" s="84"/>
-    </row>
-    <row r="384" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N384" s="84"/>
-    </row>
-    <row r="385" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N385" s="84"/>
-    </row>
-    <row r="386" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N386" s="84"/>
-    </row>
-    <row r="387" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N387" s="84"/>
-    </row>
-    <row r="388" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N388" s="84"/>
-    </row>
-    <row r="389" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N389" s="84"/>
-    </row>
-    <row r="390" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N390" s="84"/>
-    </row>
-    <row r="391" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N391" s="84"/>
-    </row>
-    <row r="392" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N392" s="84"/>
-    </row>
-    <row r="393" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N393" s="84"/>
-    </row>
-    <row r="394" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N394" s="84"/>
-    </row>
-    <row r="395" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N395" s="84"/>
-    </row>
-    <row r="396" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N396" s="84"/>
-    </row>
-    <row r="397" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N397" s="84"/>
-    </row>
-    <row r="398" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N398" s="84"/>
-    </row>
-    <row r="399" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N399" s="84"/>
-    </row>
-    <row r="400" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N400" s="84"/>
-    </row>
-    <row r="401" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N401" s="84"/>
-    </row>
-    <row r="402" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N402" s="84"/>
-    </row>
-    <row r="403" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N403" s="84"/>
-    </row>
-    <row r="404" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N404" s="84"/>
-    </row>
-    <row r="405" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N405" s="84"/>
-    </row>
-    <row r="406" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N406" s="84"/>
-    </row>
-    <row r="407" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N407" s="84"/>
-    </row>
-    <row r="408" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N408" s="84"/>
-    </row>
-    <row r="409" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N409" s="84"/>
-    </row>
-    <row r="410" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N410" s="84"/>
-    </row>
-    <row r="411" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N411" s="84"/>
-    </row>
-    <row r="412" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N412" s="84"/>
-    </row>
-    <row r="413" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N413" s="84"/>
-    </row>
-    <row r="414" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N414" s="84"/>
-    </row>
-    <row r="415" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N415" s="84"/>
-    </row>
-    <row r="416" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N416" s="84"/>
-    </row>
-    <row r="417" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N417" s="84"/>
-    </row>
-    <row r="418" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N418" s="84"/>
-    </row>
-    <row r="419" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N419" s="84"/>
-    </row>
-    <row r="420" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N420" s="84"/>
-    </row>
-    <row r="421" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N421" s="84"/>
-    </row>
-    <row r="422" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N422" s="84"/>
-    </row>
-    <row r="423" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N423" s="84"/>
-    </row>
-    <row r="424" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N424" s="84"/>
-    </row>
-    <row r="425" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N425" s="84"/>
-    </row>
-    <row r="426" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N426" s="84"/>
-    </row>
-    <row r="427" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N427" s="84"/>
-    </row>
-    <row r="428" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N428" s="84"/>
-    </row>
-    <row r="429" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N429" s="84"/>
-    </row>
-    <row r="430" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N430" s="84"/>
-    </row>
-    <row r="431" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N431" s="84"/>
-    </row>
-    <row r="432" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N432" s="84"/>
-    </row>
-    <row r="433" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N433" s="84"/>
-    </row>
-    <row r="434" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N434" s="84"/>
-    </row>
-    <row r="435" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N435" s="84"/>
-    </row>
-    <row r="436" spans="14:14" x14ac:dyDescent="0.3">
-      <c r="N436" s="83"/>
-    </row>
-    <row r="437" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N437" s="84"/>
-    </row>
-    <row r="438" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N438" s="84"/>
-    </row>
-    <row r="439" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N439" s="84"/>
-    </row>
-    <row r="440" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N440" s="84"/>
-    </row>
-    <row r="441" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N441" s="84"/>
-    </row>
-    <row r="442" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N442" s="84"/>
-    </row>
-    <row r="443" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N443" s="84"/>
-    </row>
-    <row r="444" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N444" s="84"/>
-    </row>
-    <row r="445" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N445" s="84"/>
-    </row>
-    <row r="446" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N446" s="84"/>
-    </row>
-    <row r="447" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N447" s="84"/>
-    </row>
-    <row r="448" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N448" s="84"/>
-    </row>
-    <row r="449" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N449" s="84"/>
-    </row>
-    <row r="450" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N450" s="84"/>
-    </row>
-    <row r="451" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N451" s="84"/>
-    </row>
-    <row r="452" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N452" s="84"/>
-    </row>
-    <row r="453" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N453" s="84"/>
-    </row>
-    <row r="454" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N454" s="84"/>
-    </row>
-    <row r="455" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N455" s="84"/>
-    </row>
-    <row r="456" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N456" s="84"/>
-    </row>
-    <row r="457" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N457" s="84"/>
-    </row>
-    <row r="458" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N458" s="84"/>
-    </row>
-    <row r="459" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N459" s="84"/>
-    </row>
-    <row r="460" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N460" s="84"/>
-    </row>
-    <row r="461" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N461" s="84"/>
-    </row>
-    <row r="462" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N462" s="84"/>
-    </row>
-    <row r="463" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N463" s="84"/>
-    </row>
-    <row r="464" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N464" s="84"/>
-    </row>
-    <row r="465" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N465" s="84"/>
-    </row>
-    <row r="466" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N466" s="84"/>
-    </row>
-    <row r="467" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N467" s="84"/>
-    </row>
-    <row r="468" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N468" s="84"/>
-    </row>
-    <row r="469" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N469" s="84"/>
-    </row>
-    <row r="470" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N470" s="84"/>
-    </row>
-    <row r="471" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N471" s="84"/>
-    </row>
-    <row r="472" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N472" s="84"/>
-    </row>
-    <row r="473" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N473" s="84"/>
-    </row>
-    <row r="474" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N474" s="84"/>
-    </row>
-    <row r="475" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N475" s="84"/>
-    </row>
-    <row r="476" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N476" s="84"/>
-    </row>
-    <row r="477" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N477" s="84"/>
-    </row>
-    <row r="478" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N478" s="84"/>
-    </row>
-    <row r="479" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N479" s="84"/>
-    </row>
-    <row r="480" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N480" s="84"/>
-    </row>
-    <row r="481" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N481" s="84"/>
-    </row>
-    <row r="482" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N482" s="84"/>
-    </row>
-    <row r="483" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N483" s="84"/>
-    </row>
-    <row r="484" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N484" s="84"/>
-    </row>
-    <row r="485" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N485" s="84"/>
-    </row>
-    <row r="486" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N486" s="84"/>
-    </row>
-    <row r="487" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N487" s="84"/>
-    </row>
-    <row r="488" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N488" s="84"/>
-    </row>
-    <row r="489" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N489" s="84"/>
-    </row>
-    <row r="490" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N490" s="84"/>
-    </row>
-    <row r="491" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N491" s="84"/>
-    </row>
-    <row r="492" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N492" s="84"/>
-    </row>
-    <row r="493" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N493" s="84"/>
-    </row>
-    <row r="494" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N494" s="84"/>
-    </row>
-    <row r="495" spans="14:14" x14ac:dyDescent="0.3">
-      <c r="N495" s="83"/>
-    </row>
-    <row r="496" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N496" s="84"/>
-    </row>
-    <row r="497" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N497" s="84"/>
-    </row>
-    <row r="498" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N498" s="84"/>
-    </row>
-    <row r="499" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N499" s="84"/>
-    </row>
-    <row r="500" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N500" s="84"/>
-    </row>
-    <row r="501" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N501" s="84"/>
-    </row>
-    <row r="502" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N502" s="84"/>
-    </row>
-    <row r="503" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N503" s="84"/>
-    </row>
-    <row r="504" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N504" s="84"/>
-    </row>
-    <row r="505" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N505" s="84"/>
-    </row>
-    <row r="506" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N506" s="84"/>
-    </row>
-    <row r="507" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N507" s="84"/>
-    </row>
-    <row r="508" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N508" s="84"/>
-    </row>
-    <row r="509" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N509" s="84"/>
-    </row>
-    <row r="510" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N510" s="84"/>
-    </row>
-    <row r="511" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N511" s="84"/>
-    </row>
-    <row r="512" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N512" s="84"/>
-    </row>
-    <row r="513" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N513" s="84"/>
-    </row>
-    <row r="514" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N514" s="84"/>
-    </row>
-    <row r="515" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N515" s="84"/>
-    </row>
-    <row r="516" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N516" s="84"/>
-    </row>
-    <row r="517" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N517" s="84"/>
-    </row>
-    <row r="518" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N518" s="84"/>
-    </row>
-    <row r="519" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N519" s="84"/>
-    </row>
-    <row r="520" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N520" s="84"/>
-    </row>
-    <row r="521" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N521" s="84"/>
-    </row>
-    <row r="522" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N522" s="84"/>
-    </row>
-    <row r="523" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N523" s="84"/>
-    </row>
-    <row r="524" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N524" s="84"/>
-    </row>
-    <row r="525" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N525" s="84"/>
-    </row>
-    <row r="526" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N526" s="84"/>
-    </row>
-    <row r="527" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N527" s="84"/>
-    </row>
-    <row r="528" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N528" s="84"/>
-    </row>
-    <row r="529" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N529" s="84"/>
-    </row>
-    <row r="530" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N530" s="84"/>
-    </row>
-    <row r="531" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N531" s="84"/>
-    </row>
-    <row r="532" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N532" s="84"/>
-    </row>
-    <row r="533" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N533" s="84"/>
-    </row>
-    <row r="534" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N534" s="84"/>
-    </row>
-    <row r="535" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N535" s="84"/>
-    </row>
-    <row r="536" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N536" s="84"/>
-    </row>
-    <row r="537" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N537" s="84"/>
-    </row>
-    <row r="538" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N538" s="84"/>
-    </row>
-    <row r="539" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N539" s="84"/>
-    </row>
-    <row r="540" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N540" s="84"/>
-    </row>
-    <row r="541" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N541" s="84"/>
-    </row>
-    <row r="542" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N542" s="84"/>
-    </row>
-    <row r="543" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N543" s="84"/>
-    </row>
-    <row r="544" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N544" s="84"/>
-    </row>
-    <row r="545" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N545" s="84"/>
-    </row>
-    <row r="546" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N546" s="84"/>
-    </row>
-    <row r="547" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N547" s="84"/>
-    </row>
-    <row r="548" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N548" s="84"/>
-    </row>
-    <row r="549" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N549" s="84"/>
-    </row>
-    <row r="550" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N550" s="84"/>
-    </row>
-    <row r="551" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N551" s="84"/>
-    </row>
-    <row r="552" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N552" s="84"/>
-    </row>
-    <row r="553" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N553" s="84"/>
-    </row>
-    <row r="554" spans="14:14" x14ac:dyDescent="0.3">
-      <c r="N554" s="83"/>
-    </row>
-    <row r="555" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N555" s="84"/>
-    </row>
-    <row r="556" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N556" s="84"/>
-    </row>
-    <row r="557" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N557" s="84"/>
-    </row>
-    <row r="558" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N558" s="84"/>
-    </row>
-    <row r="559" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N559" s="84"/>
-    </row>
-    <row r="560" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N560" s="84"/>
-    </row>
-    <row r="561" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N561" s="84"/>
-    </row>
-    <row r="562" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N562" s="84"/>
-    </row>
-    <row r="563" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N563" s="84"/>
-    </row>
-    <row r="564" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N564" s="84"/>
-    </row>
-    <row r="565" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N565" s="84"/>
-    </row>
-    <row r="566" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N566" s="84"/>
-    </row>
-    <row r="567" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N567" s="84"/>
-    </row>
-    <row r="568" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N568" s="84"/>
-    </row>
-    <row r="569" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N569" s="84"/>
-    </row>
-    <row r="570" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N570" s="84"/>
-    </row>
-    <row r="571" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N571" s="84"/>
-    </row>
-    <row r="572" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N572" s="84"/>
-    </row>
-    <row r="573" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N573" s="84"/>
-    </row>
-    <row r="574" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N574" s="84"/>
-    </row>
-    <row r="575" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N575" s="84"/>
-    </row>
-    <row r="576" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N576" s="84"/>
-    </row>
-    <row r="577" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N577" s="84"/>
-    </row>
-    <row r="578" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N578" s="84"/>
-    </row>
-    <row r="579" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N579" s="84"/>
-    </row>
-    <row r="580" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N580" s="84"/>
-    </row>
-    <row r="581" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N581" s="84"/>
-    </row>
-    <row r="582" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N582" s="84"/>
-    </row>
-    <row r="583" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N583" s="84"/>
-    </row>
-    <row r="584" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N584" s="84"/>
-    </row>
-    <row r="585" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N585" s="84"/>
-    </row>
-    <row r="586" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N586" s="84"/>
-    </row>
-    <row r="587" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N587" s="84"/>
-    </row>
-    <row r="588" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N588" s="84"/>
-    </row>
-    <row r="589" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N589" s="84"/>
-    </row>
-    <row r="590" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N590" s="84"/>
-    </row>
-    <row r="591" spans="14:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="N591" s="84"/>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="I2:K3"/>
-    <mergeCell ref="L2:L4"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:R1"/>
   <sheetFormatPr defaultColWidth="8" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>